<commit_message>
Update RSI screener report 2026-08-15 11:52 UTC
</commit_message>
<xml_diff>
--- a/docs/nifty500_rsi_report.xlsx
+++ b/docs/nifty500_rsi_report.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -463,6 +463,82 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>POWERGRID</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>266.05</v>
+      </c>
+      <c r="C2" t="n">
+        <v>35.92</v>
+      </c>
+      <c r="D2" t="n">
+        <v>46.67</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-17.09</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>HINDUNILVR</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2077</v>
+      </c>
+      <c r="C3" t="n">
+        <v>37.4</v>
+      </c>
+      <c r="D3" t="n">
+        <v>40.85</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-22.86</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ONGC</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>236.4</v>
+      </c>
+      <c r="C4" t="n">
+        <v>39.23</v>
+      </c>
+      <c r="D4" t="n">
+        <v>46.99</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-21.57</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>NTPC</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>340</v>
+      </c>
+      <c r="C5" t="n">
+        <v>39.76</v>
+      </c>
+      <c r="D5" t="n">
+        <v>49.94</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-17.11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update RSI screener report 2026-08-16 05:37 UTC
</commit_message>
<xml_diff>
--- a/docs/nifty500_rsi_report.xlsx
+++ b/docs/nifty500_rsi_report.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -520,25 +520,6 @@
         <v>-21.57</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>NTPC</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>340</v>
-      </c>
-      <c r="C5" t="n">
-        <v>39.76</v>
-      </c>
-      <c r="D5" t="n">
-        <v>49.94</v>
-      </c>
-      <c r="E5" t="n">
-        <v>-17.11</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update RSI screener report 2026-08-16 05:42 UTC
</commit_message>
<xml_diff>
--- a/docs/nifty500_rsi_report.xlsx
+++ b/docs/nifty500_rsi_report.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -520,6 +520,25 @@
         <v>-21.57</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>NTPC</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>340</v>
+      </c>
+      <c r="C5" t="n">
+        <v>39.76</v>
+      </c>
+      <c r="D5" t="n">
+        <v>49.94</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-17.11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update RSI screener report 2026-08-16 06:13 UTC
</commit_message>
<xml_diff>
--- a/docs/nifty500_rsi_report.xlsx
+++ b/docs/nifty500_rsi_report.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -463,82 +463,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>POWERGRID</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>266.05</v>
-      </c>
-      <c r="C2" t="n">
-        <v>35.92</v>
-      </c>
-      <c r="D2" t="n">
-        <v>46.67</v>
-      </c>
-      <c r="E2" t="n">
-        <v>-17.09</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>HINDUNILVR</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>2077</v>
-      </c>
-      <c r="C3" t="n">
-        <v>37.4</v>
-      </c>
-      <c r="D3" t="n">
-        <v>40.85</v>
-      </c>
-      <c r="E3" t="n">
-        <v>-22.86</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>ONGC</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>236.4</v>
-      </c>
-      <c r="C4" t="n">
-        <v>39.23</v>
-      </c>
-      <c r="D4" t="n">
-        <v>46.99</v>
-      </c>
-      <c r="E4" t="n">
-        <v>-21.57</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>NTPC</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>340</v>
-      </c>
-      <c r="C5" t="n">
-        <v>39.76</v>
-      </c>
-      <c r="D5" t="n">
-        <v>49.94</v>
-      </c>
-      <c r="E5" t="n">
-        <v>-17.11</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update RSI screener report 2026-08-16 06:16 UTC
</commit_message>
<xml_diff>
--- a/docs/nifty500_rsi_report.xlsx
+++ b/docs/nifty500_rsi_report.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -463,6 +463,82 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>POWERGRID</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>266.05</v>
+      </c>
+      <c r="C2" t="n">
+        <v>35.92</v>
+      </c>
+      <c r="D2" t="n">
+        <v>46.67</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-17.09</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>HINDUNILVR</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2077</v>
+      </c>
+      <c r="C3" t="n">
+        <v>37.4</v>
+      </c>
+      <c r="D3" t="n">
+        <v>40.85</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-22.86</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ONGC</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>236.4</v>
+      </c>
+      <c r="C4" t="n">
+        <v>39.23</v>
+      </c>
+      <c r="D4" t="n">
+        <v>46.99</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-21.57</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>NTPC</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>340</v>
+      </c>
+      <c r="C5" t="n">
+        <v>39.76</v>
+      </c>
+      <c r="D5" t="n">
+        <v>49.94</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-17.11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update RSI screener report 2026-08-17 04:02 UTC
</commit_message>
<xml_diff>
--- a/docs/nifty500_rsi_report.xlsx
+++ b/docs/nifty500_rsi_report.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -466,77 +466,172 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>266.05</v>
+        <v>276.1</v>
       </c>
       <c r="C2" t="n">
-        <v>35.92</v>
+        <v>32.55</v>
       </c>
       <c r="D2" t="n">
-        <v>46.67</v>
+        <v>30.94</v>
       </c>
       <c r="E2" t="n">
-        <v>-17.09</v>
+        <v>-34.51</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2077</v>
+        <v>726.2</v>
       </c>
       <c r="C3" t="n">
-        <v>37.4</v>
+        <v>33.63</v>
       </c>
       <c r="D3" t="n">
-        <v>40.85</v>
+        <v>38.47</v>
       </c>
       <c r="E3" t="n">
-        <v>-22.86</v>
+        <v>-28.06</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>236.4</v>
+        <v>540.25</v>
       </c>
       <c r="C4" t="n">
-        <v>39.23</v>
+        <v>33.66</v>
       </c>
       <c r="D4" t="n">
-        <v>46.99</v>
+        <v>36.16</v>
       </c>
       <c r="E4" t="n">
-        <v>-21.57</v>
+        <v>-32.18</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>POWERGRID</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>266.1</v>
+      </c>
+      <c r="C5" t="n">
+        <v>35.96</v>
+      </c>
+      <c r="D5" t="n">
+        <v>46.68</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-17.08</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>HINDUNILVR</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2062.7</v>
+      </c>
+      <c r="C6" t="n">
+        <v>36.32</v>
+      </c>
+      <c r="D6" t="n">
+        <v>40.45</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-23.39</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>WIPRO</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>181.59</v>
+      </c>
+      <c r="C7" t="n">
+        <v>38.53</v>
+      </c>
+      <c r="D7" t="n">
+        <v>38.18</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-33.4</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>NTPC</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>340</v>
-      </c>
-      <c r="C5" t="n">
-        <v>39.76</v>
-      </c>
-      <c r="D5" t="n">
-        <v>49.94</v>
-      </c>
-      <c r="E5" t="n">
-        <v>-17.11</v>
+      <c r="B8" t="n">
+        <v>338.5</v>
+      </c>
+      <c r="C8" t="n">
+        <v>39.13</v>
+      </c>
+      <c r="D8" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-17.48</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>COALINDIA</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>406.3</v>
+      </c>
+      <c r="C9" t="n">
+        <v>39.83</v>
+      </c>
+      <c r="D9" t="n">
+        <v>50.15</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-15.64</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ONGC</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>237.32</v>
+      </c>
+      <c r="C10" t="n">
+        <v>39.85</v>
+      </c>
+      <c r="D10" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-21.26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update RSI screener report 2026-08-17 05:27 UTC
</commit_message>
<xml_diff>
--- a/docs/nifty500_rsi_report.xlsx
+++ b/docs/nifty500_rsi_report.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -470,168 +470,301 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>276.1</v>
+        <v>275.5</v>
       </c>
       <c r="C2" t="n">
-        <v>32.55</v>
+        <v>32.3</v>
       </c>
       <c r="D2" t="n">
-        <v>30.94</v>
+        <v>30.87</v>
       </c>
       <c r="E2" t="n">
-        <v>-34.51</v>
+        <v>-34.65</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>IRFC</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>726.2</v>
+        <v>86.59</v>
       </c>
       <c r="C3" t="n">
-        <v>33.63</v>
+        <v>32.4</v>
       </c>
       <c r="D3" t="n">
-        <v>38.47</v>
+        <v>40.08</v>
       </c>
       <c r="E3" t="n">
-        <v>-28.06</v>
+        <v>-35.21</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>GODREJCP</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>540.25</v>
+        <v>928</v>
       </c>
       <c r="C4" t="n">
-        <v>33.66</v>
+        <v>32.9</v>
       </c>
       <c r="D4" t="n">
-        <v>36.16</v>
+        <v>40.5</v>
       </c>
       <c r="E4" t="n">
-        <v>-32.18</v>
+        <v>-27.71</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>VEDL</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>266.1</v>
+        <v>269.2</v>
       </c>
       <c r="C5" t="n">
-        <v>35.96</v>
+        <v>33.04</v>
       </c>
       <c r="D5" t="n">
-        <v>46.68</v>
+        <v>39.85</v>
       </c>
       <c r="E5" t="n">
-        <v>-17.08</v>
+        <v>-65.81999999999999</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2062.7</v>
+        <v>725</v>
       </c>
       <c r="C6" t="n">
-        <v>36.32</v>
+        <v>33.45</v>
       </c>
       <c r="D6" t="n">
-        <v>40.45</v>
+        <v>38.39</v>
       </c>
       <c r="E6" t="n">
-        <v>-23.39</v>
+        <v>-28.18</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>181.59</v>
+        <v>542.75</v>
       </c>
       <c r="C7" t="n">
-        <v>38.53</v>
+        <v>34.52</v>
       </c>
       <c r="D7" t="n">
-        <v>38.18</v>
+        <v>36.37</v>
       </c>
       <c r="E7" t="n">
-        <v>-33.4</v>
+        <v>-31.86</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>338.5</v>
+        <v>266</v>
       </c>
       <c r="C8" t="n">
-        <v>39.13</v>
+        <v>35.9</v>
       </c>
       <c r="D8" t="n">
-        <v>49.6</v>
+        <v>46.66</v>
       </c>
       <c r="E8" t="n">
-        <v>-17.48</v>
+        <v>-17.11</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>406.3</v>
+        <v>2060.9</v>
       </c>
       <c r="C9" t="n">
-        <v>39.83</v>
+        <v>36.19</v>
       </c>
       <c r="D9" t="n">
-        <v>50.15</v>
+        <v>40.4</v>
       </c>
       <c r="E9" t="n">
-        <v>-15.64</v>
+        <v>-23.46</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>AMBUJACEM</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>412.1</v>
+      </c>
+      <c r="C10" t="n">
+        <v>36.6</v>
+      </c>
+      <c r="D10" t="n">
+        <v>37.75</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-30.44</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>PFC</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>375</v>
+      </c>
+      <c r="C11" t="n">
+        <v>38.04</v>
+      </c>
+      <c r="D11" t="n">
+        <v>47.79</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-22.1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>MUTHOOTFIN</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>2869.8</v>
+      </c>
+      <c r="C12" t="n">
+        <v>38.09</v>
+      </c>
+      <c r="D12" t="n">
+        <v>52.81</v>
+      </c>
+      <c r="E12" t="n">
+        <v>-29.86</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>WIPRO</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>181.56</v>
+      </c>
+      <c r="C13" t="n">
+        <v>38.52</v>
+      </c>
+      <c r="D13" t="n">
+        <v>38.18</v>
+      </c>
+      <c r="E13" t="n">
+        <v>-33.41</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>VBL</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>436.1</v>
+      </c>
+      <c r="C14" t="n">
+        <v>38.74</v>
+      </c>
+      <c r="D14" t="n">
+        <v>46.25</v>
+      </c>
+      <c r="E14" t="n">
+        <v>-19.84</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>NTPC</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>339.1</v>
+      </c>
+      <c r="C15" t="n">
+        <v>39.38</v>
+      </c>
+      <c r="D15" t="n">
+        <v>49.74</v>
+      </c>
+      <c r="E15" t="n">
+        <v>-17.33</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>BANKBARODA</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>244.68</v>
+      </c>
+      <c r="C16" t="n">
+        <v>39.87</v>
+      </c>
+      <c r="D16" t="n">
+        <v>48.29</v>
+      </c>
+      <c r="E16" t="n">
+        <v>-24.59</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>ONGC</t>
         </is>
       </c>
-      <c r="B10" t="n">
-        <v>237.32</v>
-      </c>
-      <c r="C10" t="n">
-        <v>39.85</v>
-      </c>
-      <c r="D10" t="n">
-        <v>47.2</v>
-      </c>
-      <c r="E10" t="n">
-        <v>-21.26</v>
+      <c r="B17" t="n">
+        <v>237.4</v>
+      </c>
+      <c r="C17" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="D17" t="n">
+        <v>47.22</v>
+      </c>
+      <c r="E17" t="n">
+        <v>-21.23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update RSI screener report 2026-08-22 04:02 UTC
</commit_message>
<xml_diff>
--- a/docs/nifty500_rsi_report.xlsx
+++ b/docs/nifty500_rsi_report.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -470,16 +470,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>275.5</v>
+        <v>269.4</v>
       </c>
       <c r="C2" t="n">
-        <v>32.3</v>
+        <v>29.98</v>
       </c>
       <c r="D2" t="n">
-        <v>30.87</v>
+        <v>30.08</v>
       </c>
       <c r="E2" t="n">
-        <v>-34.65</v>
+        <v>-36.1</v>
       </c>
     </row>
     <row r="3">
@@ -489,16 +489,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>86.59</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="C3" t="n">
-        <v>32.4</v>
+        <v>32.21</v>
       </c>
       <c r="D3" t="n">
-        <v>40.08</v>
+        <v>40.02</v>
       </c>
       <c r="E3" t="n">
-        <v>-35.21</v>
+        <v>-35.35</v>
       </c>
     </row>
     <row r="4">
@@ -508,168 +508,168 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>928</v>
+        <v>933</v>
       </c>
       <c r="C4" t="n">
-        <v>32.9</v>
+        <v>33.32</v>
       </c>
       <c r="D4" t="n">
-        <v>40.5</v>
+        <v>40.7</v>
       </c>
       <c r="E4" t="n">
-        <v>-27.71</v>
+        <v>-27.33</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>VEDL</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>269.2</v>
+        <v>726.95</v>
       </c>
       <c r="C5" t="n">
-        <v>33.04</v>
+        <v>33.74</v>
       </c>
       <c r="D5" t="n">
-        <v>39.85</v>
+        <v>38.52</v>
       </c>
       <c r="E5" t="n">
-        <v>-65.81999999999999</v>
+        <v>-27.99</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>725</v>
+        <v>2028</v>
       </c>
       <c r="C6" t="n">
-        <v>33.45</v>
+        <v>33.94</v>
       </c>
       <c r="D6" t="n">
-        <v>38.39</v>
+        <v>39.52</v>
       </c>
       <c r="E6" t="n">
-        <v>-28.18</v>
+        <v>-24.68</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>VEDL</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>542.75</v>
+        <v>279</v>
       </c>
       <c r="C7" t="n">
-        <v>34.52</v>
+        <v>34.78</v>
       </c>
       <c r="D7" t="n">
-        <v>36.37</v>
+        <v>40.59</v>
       </c>
       <c r="E7" t="n">
-        <v>-31.86</v>
+        <v>-64.56999999999999</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>PFC</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>266</v>
+        <v>363</v>
       </c>
       <c r="C8" t="n">
-        <v>35.9</v>
+        <v>35.53</v>
       </c>
       <c r="D8" t="n">
-        <v>46.66</v>
+        <v>46.36</v>
       </c>
       <c r="E8" t="n">
-        <v>-17.11</v>
+        <v>-24.59</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>AMBUJACEM</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2060.9</v>
+        <v>414.5</v>
       </c>
       <c r="C9" t="n">
-        <v>36.19</v>
+        <v>37.22</v>
       </c>
       <c r="D9" t="n">
-        <v>40.4</v>
+        <v>37.99</v>
       </c>
       <c r="E9" t="n">
-        <v>-23.46</v>
+        <v>-29.94</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AMBUJACEM</t>
+          <t>VBL</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>412.1</v>
+        <v>430.1</v>
       </c>
       <c r="C10" t="n">
-        <v>36.6</v>
+        <v>37.29</v>
       </c>
       <c r="D10" t="n">
-        <v>37.75</v>
+        <v>45.73</v>
       </c>
       <c r="E10" t="n">
-        <v>-30.44</v>
+        <v>-20.94</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PFC</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>375</v>
+        <v>317.9</v>
       </c>
       <c r="C11" t="n">
-        <v>38.04</v>
+        <v>37.48</v>
       </c>
       <c r="D11" t="n">
-        <v>47.79</v>
+        <v>35.14</v>
       </c>
       <c r="E11" t="n">
-        <v>-22.1</v>
+        <v>-55.82</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MUTHOOTFIN</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2869.8</v>
+        <v>1049</v>
       </c>
       <c r="C12" t="n">
-        <v>38.09</v>
+        <v>37.53</v>
       </c>
       <c r="D12" t="n">
-        <v>52.81</v>
+        <v>48.32</v>
       </c>
       <c r="E12" t="n">
-        <v>-29.86</v>
+        <v>-17.47</v>
       </c>
     </row>
     <row r="13">
@@ -679,92 +679,111 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>181.56</v>
+        <v>180.79</v>
       </c>
       <c r="C13" t="n">
-        <v>38.52</v>
+        <v>38.06</v>
       </c>
       <c r="D13" t="n">
-        <v>38.18</v>
+        <v>38.03</v>
       </c>
       <c r="E13" t="n">
-        <v>-33.41</v>
+        <v>-33.7</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>VBL</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>436.1</v>
+        <v>554.8</v>
       </c>
       <c r="C14" t="n">
-        <v>38.74</v>
+        <v>38.35</v>
       </c>
       <c r="D14" t="n">
-        <v>46.25</v>
+        <v>37.76</v>
       </c>
       <c r="E14" t="n">
-        <v>-19.84</v>
+        <v>-30.25</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>339.1</v>
+        <v>236.4</v>
       </c>
       <c r="C15" t="n">
-        <v>39.38</v>
+        <v>39.23</v>
       </c>
       <c r="D15" t="n">
-        <v>49.74</v>
+        <v>46.99</v>
       </c>
       <c r="E15" t="n">
-        <v>-17.33</v>
+        <v>-21.57</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>BANKBARODA</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>244.68</v>
+        <v>405.2</v>
       </c>
       <c r="C16" t="n">
-        <v>39.87</v>
+        <v>39.5</v>
       </c>
       <c r="D16" t="n">
-        <v>48.29</v>
+        <v>49.94</v>
       </c>
       <c r="E16" t="n">
-        <v>-24.59</v>
+        <v>-15.87</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>RECLTD</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>237.4</v>
+        <v>326.65</v>
       </c>
       <c r="C17" t="n">
-        <v>39.9</v>
+        <v>39.68</v>
       </c>
       <c r="D17" t="n">
-        <v>47.22</v>
+        <v>44.13</v>
       </c>
       <c r="E17" t="n">
-        <v>-21.23</v>
+        <v>-15.53</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>NTPC</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>340</v>
+      </c>
+      <c r="C18" t="n">
+        <v>39.76</v>
+      </c>
+      <c r="D18" t="n">
+        <v>49.94</v>
+      </c>
+      <c r="E18" t="n">
+        <v>-17.11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update RSI screener report 2026-08-29 10:16 UTC
</commit_message>
<xml_diff>
--- a/docs/nifty500_rsi_report.xlsx
+++ b/docs/nifty500_rsi_report.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -470,16 +470,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>269.4</v>
+        <v>269</v>
       </c>
       <c r="C2" t="n">
-        <v>29.98</v>
+        <v>29.83</v>
       </c>
       <c r="D2" t="n">
-        <v>30.08</v>
+        <v>30.03</v>
       </c>
       <c r="E2" t="n">
-        <v>-36.1</v>
+        <v>-36.2</v>
       </c>
     </row>
     <row r="3">
@@ -489,54 +489,54 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>86.40000000000001</v>
+        <v>84.65000000000001</v>
       </c>
       <c r="C3" t="n">
-        <v>32.21</v>
+        <v>30.46</v>
       </c>
       <c r="D3" t="n">
-        <v>40.02</v>
+        <v>39.47</v>
       </c>
       <c r="E3" t="n">
-        <v>-35.35</v>
+        <v>-36.66</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GODREJCP</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>933</v>
+        <v>711</v>
       </c>
       <c r="C4" t="n">
-        <v>33.32</v>
+        <v>31.41</v>
       </c>
       <c r="D4" t="n">
-        <v>40.7</v>
+        <v>37.45</v>
       </c>
       <c r="E4" t="n">
-        <v>-27.33</v>
+        <v>-29.57</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>GODREJCP</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>726.95</v>
+        <v>923</v>
       </c>
       <c r="C5" t="n">
-        <v>33.74</v>
+        <v>32.44</v>
       </c>
       <c r="D5" t="n">
-        <v>38.52</v>
+        <v>40.31</v>
       </c>
       <c r="E5" t="n">
-        <v>-27.99</v>
+        <v>-28.1</v>
       </c>
     </row>
     <row r="6">
@@ -546,244 +546,301 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2028</v>
+        <v>2009</v>
       </c>
       <c r="C6" t="n">
-        <v>33.94</v>
+        <v>32.73</v>
       </c>
       <c r="D6" t="n">
-        <v>39.52</v>
+        <v>39.03</v>
       </c>
       <c r="E6" t="n">
-        <v>-24.68</v>
+        <v>-24.95</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>VEDL</t>
+          <t>PFC</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>279</v>
+        <v>355.85</v>
       </c>
       <c r="C7" t="n">
-        <v>34.78</v>
+        <v>34.08</v>
       </c>
       <c r="D7" t="n">
-        <v>40.59</v>
+        <v>45.54</v>
       </c>
       <c r="E7" t="n">
-        <v>-64.56999999999999</v>
+        <v>-26.08</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PFC</t>
+          <t>VBL</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>363</v>
+        <v>418.75</v>
       </c>
       <c r="C8" t="n">
-        <v>35.53</v>
+        <v>34.89</v>
       </c>
       <c r="D8" t="n">
-        <v>46.36</v>
+        <v>44.78</v>
       </c>
       <c r="E8" t="n">
-        <v>-24.59</v>
+        <v>-23.03</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AMBUJACEM</t>
+          <t>VEDL</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>414.5</v>
+        <v>281</v>
       </c>
       <c r="C9" t="n">
-        <v>37.22</v>
+        <v>35.16</v>
       </c>
       <c r="D9" t="n">
-        <v>37.99</v>
+        <v>40.73</v>
       </c>
       <c r="E9" t="n">
-        <v>-29.94</v>
+        <v>-64.31999999999999</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>VBL</t>
+          <t>TATAPOWER</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>430.1</v>
+        <v>352</v>
       </c>
       <c r="C10" t="n">
-        <v>37.29</v>
+        <v>35.47</v>
       </c>
       <c r="D10" t="n">
-        <v>45.73</v>
+        <v>45.61</v>
       </c>
       <c r="E10" t="n">
-        <v>-20.94</v>
+        <v>-23.78</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>WIPRO</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>317.9</v>
+        <v>176.4</v>
       </c>
       <c r="C11" t="n">
-        <v>37.48</v>
+        <v>35.49</v>
       </c>
       <c r="D11" t="n">
-        <v>35.14</v>
+        <v>37.21</v>
       </c>
       <c r="E11" t="n">
-        <v>-55.82</v>
+        <v>-35.31</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1049</v>
+        <v>330.9</v>
       </c>
       <c r="C12" t="n">
-        <v>37.53</v>
+        <v>35.97</v>
       </c>
       <c r="D12" t="n">
-        <v>48.32</v>
+        <v>47.94</v>
       </c>
       <c r="E12" t="n">
-        <v>-17.47</v>
+        <v>-19.33</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>AMBUJACEM</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>180.79</v>
+        <v>411.05</v>
       </c>
       <c r="C13" t="n">
-        <v>38.06</v>
+        <v>36.27</v>
       </c>
       <c r="D13" t="n">
-        <v>38.03</v>
+        <v>37.64</v>
       </c>
       <c r="E13" t="n">
-        <v>-33.7</v>
+        <v>-30.52</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>554.8</v>
+        <v>1042</v>
       </c>
       <c r="C14" t="n">
-        <v>38.35</v>
+        <v>36.52</v>
       </c>
       <c r="D14" t="n">
-        <v>37.76</v>
+        <v>47.87</v>
       </c>
       <c r="E14" t="n">
-        <v>-30.25</v>
+        <v>-18.02</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>236.4</v>
+        <v>548</v>
       </c>
       <c r="C15" t="n">
-        <v>39.23</v>
+        <v>37.03</v>
       </c>
       <c r="D15" t="n">
-        <v>46.99</v>
+        <v>36.81</v>
       </c>
       <c r="E15" t="n">
-        <v>-21.57</v>
+        <v>-30.44</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>405.2</v>
+        <v>316</v>
       </c>
       <c r="C16" t="n">
-        <v>39.5</v>
+        <v>37.07</v>
       </c>
       <c r="D16" t="n">
-        <v>49.94</v>
+        <v>35.05</v>
       </c>
       <c r="E16" t="n">
-        <v>-15.87</v>
+        <v>-56.08</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>RECLTD</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>326.65</v>
+        <v>264.9</v>
       </c>
       <c r="C17" t="n">
-        <v>39.68</v>
+        <v>37.23</v>
       </c>
       <c r="D17" t="n">
-        <v>44.13</v>
+        <v>46.42</v>
       </c>
       <c r="E17" t="n">
-        <v>-15.53</v>
+        <v>-17.45</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>340</v>
+        <v>232</v>
       </c>
       <c r="C18" t="n">
-        <v>39.76</v>
+        <v>37.26</v>
       </c>
       <c r="D18" t="n">
-        <v>49.94</v>
+        <v>46</v>
       </c>
       <c r="E18" t="n">
-        <v>-17.11</v>
+        <v>-23.03</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>COALINDIA</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>400</v>
+      </c>
+      <c r="C19" t="n">
+        <v>37.86</v>
+      </c>
+      <c r="D19" t="n">
+        <v>49.01</v>
+      </c>
+      <c r="E19" t="n">
+        <v>-16.95</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>RECLTD</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>320.9</v>
+      </c>
+      <c r="C20" t="n">
+        <v>38</v>
+      </c>
+      <c r="D20" t="n">
+        <v>43.48</v>
+      </c>
+      <c r="E20" t="n">
+        <v>-17.02</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>BANKBARODA</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>241</v>
+      </c>
+      <c r="C21" t="n">
+        <v>38.21</v>
+      </c>
+      <c r="D21" t="n">
+        <v>47.42</v>
+      </c>
+      <c r="E21" t="n">
+        <v>-25.72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update RSI screener report 2026-09-05 07:46 UTC
</commit_message>
<xml_diff>
--- a/docs/nifty500_rsi_report.xlsx
+++ b/docs/nifty500_rsi_report.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -470,111 +470,111 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>269</v>
+        <v>264.1</v>
       </c>
       <c r="C2" t="n">
-        <v>29.83</v>
+        <v>28.04</v>
       </c>
       <c r="D2" t="n">
-        <v>30.03</v>
+        <v>30.95</v>
       </c>
       <c r="E2" t="n">
-        <v>-36.2</v>
+        <v>-37.36</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>IRFC</t>
+          <t>GODREJCP</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>84.65000000000001</v>
+        <v>878</v>
       </c>
       <c r="C3" t="n">
-        <v>30.46</v>
+        <v>28.82</v>
       </c>
       <c r="D3" t="n">
-        <v>39.47</v>
+        <v>38.59</v>
       </c>
       <c r="E3" t="n">
-        <v>-36.66</v>
+        <v>-30.68</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>IRFC</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>711</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="C4" t="n">
-        <v>31.41</v>
+        <v>29.29</v>
       </c>
       <c r="D4" t="n">
-        <v>37.45</v>
+        <v>39.1</v>
       </c>
       <c r="E4" t="n">
-        <v>-29.57</v>
+        <v>-37.59</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GODREJCP</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>923</v>
+        <v>1973.4</v>
       </c>
       <c r="C5" t="n">
-        <v>32.44</v>
+        <v>30.43</v>
       </c>
       <c r="D5" t="n">
-        <v>40.31</v>
+        <v>38.25</v>
       </c>
       <c r="E5" t="n">
-        <v>-28.1</v>
+        <v>-26</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2009</v>
+        <v>712.1</v>
       </c>
       <c r="C6" t="n">
-        <v>32.73</v>
+        <v>31.47</v>
       </c>
       <c r="D6" t="n">
-        <v>39.03</v>
+        <v>37.68</v>
       </c>
       <c r="E6" t="n">
-        <v>-24.95</v>
+        <v>-29.46</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PFC</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>355.85</v>
+        <v>1010</v>
       </c>
       <c r="C7" t="n">
-        <v>34.08</v>
+        <v>32.29</v>
       </c>
       <c r="D7" t="n">
-        <v>45.54</v>
+        <v>45.79</v>
       </c>
       <c r="E7" t="n">
-        <v>-26.08</v>
+        <v>-20.54</v>
       </c>
     </row>
     <row r="8">
@@ -584,225 +584,225 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>418.75</v>
+        <v>407.6</v>
       </c>
       <c r="C8" t="n">
-        <v>34.89</v>
+        <v>32.73</v>
       </c>
       <c r="D8" t="n">
-        <v>44.78</v>
+        <v>44.1</v>
       </c>
       <c r="E8" t="n">
-        <v>-23.03</v>
+        <v>-25.08</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>VEDL</t>
+          <t>AMBUJACEM</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>281</v>
+        <v>405</v>
       </c>
       <c r="C9" t="n">
-        <v>35.16</v>
+        <v>34.59</v>
       </c>
       <c r="D9" t="n">
-        <v>40.73</v>
+        <v>37.35</v>
       </c>
       <c r="E9" t="n">
-        <v>-64.31999999999999</v>
+        <v>-31.54</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TATAPOWER</t>
+          <t>PFC</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>352</v>
+        <v>355.6</v>
       </c>
       <c r="C10" t="n">
-        <v>35.47</v>
+        <v>34.76</v>
       </c>
       <c r="D10" t="n">
-        <v>45.61</v>
+        <v>46.08</v>
       </c>
       <c r="E10" t="n">
-        <v>-23.78</v>
+        <v>-26.13</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>VEDL</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>176.4</v>
+        <v>272.1</v>
       </c>
       <c r="C11" t="n">
-        <v>35.49</v>
+        <v>34.76</v>
       </c>
       <c r="D11" t="n">
-        <v>37.21</v>
+        <v>40.2</v>
       </c>
       <c r="E11" t="n">
-        <v>-35.31</v>
+        <v>-65.45</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>WIPRO</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>330.9</v>
+        <v>176.4</v>
       </c>
       <c r="C12" t="n">
-        <v>35.97</v>
+        <v>35.37</v>
       </c>
       <c r="D12" t="n">
-        <v>47.94</v>
+        <v>37.2</v>
       </c>
       <c r="E12" t="n">
-        <v>-19.33</v>
+        <v>-35.31</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AMBUJACEM</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>411.05</v>
+        <v>311.5</v>
       </c>
       <c r="C13" t="n">
-        <v>36.27</v>
+        <v>36.23</v>
       </c>
       <c r="D13" t="n">
-        <v>37.64</v>
+        <v>34.96</v>
       </c>
       <c r="E13" t="n">
-        <v>-30.52</v>
+        <v>-56.71</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1042</v>
+        <v>5130</v>
       </c>
       <c r="C14" t="n">
-        <v>36.52</v>
+        <v>36.27</v>
       </c>
       <c r="D14" t="n">
-        <v>47.87</v>
+        <v>46.07</v>
       </c>
       <c r="E14" t="n">
-        <v>-18.02</v>
+        <v>-18.58</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>548</v>
+        <v>5130</v>
       </c>
       <c r="C15" t="n">
-        <v>37.03</v>
+        <v>36.27</v>
       </c>
       <c r="D15" t="n">
-        <v>36.81</v>
+        <v>46.07</v>
       </c>
       <c r="E15" t="n">
-        <v>-30.44</v>
+        <v>-18.58</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>316</v>
+        <v>546.4</v>
       </c>
       <c r="C16" t="n">
-        <v>37.07</v>
+        <v>36.71</v>
       </c>
       <c r="D16" t="n">
-        <v>35.05</v>
+        <v>36.89</v>
       </c>
       <c r="E16" t="n">
-        <v>-56.08</v>
+        <v>-30.64</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>BANKBARODA</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>264.9</v>
+        <v>239</v>
       </c>
       <c r="C17" t="n">
-        <v>37.23</v>
+        <v>37.32</v>
       </c>
       <c r="D17" t="n">
-        <v>46.42</v>
+        <v>47</v>
       </c>
       <c r="E17" t="n">
-        <v>-17.45</v>
+        <v>-26.34</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>232</v>
+        <v>332.5</v>
       </c>
       <c r="C18" t="n">
-        <v>37.26</v>
+        <v>37.37</v>
       </c>
       <c r="D18" t="n">
-        <v>46</v>
+        <v>48.44</v>
       </c>
       <c r="E18" t="n">
-        <v>-23.03</v>
+        <v>-18.94</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>400</v>
+        <v>266</v>
       </c>
       <c r="C19" t="n">
-        <v>37.86</v>
+        <v>37.72</v>
       </c>
       <c r="D19" t="n">
-        <v>49.01</v>
+        <v>46.78</v>
       </c>
       <c r="E19" t="n">
-        <v>-16.95</v>
+        <v>-17.11</v>
       </c>
     </row>
     <row r="20">
@@ -812,35 +812,92 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>320.9</v>
+        <v>318.7</v>
       </c>
       <c r="C20" t="n">
-        <v>38</v>
+        <v>37.79</v>
       </c>
       <c r="D20" t="n">
-        <v>43.48</v>
+        <v>43.2</v>
       </c>
       <c r="E20" t="n">
-        <v>-17.02</v>
+        <v>-17.58</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>BANKBARODA</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>241</v>
+        <v>12694</v>
       </c>
       <c r="C21" t="n">
-        <v>38.21</v>
+        <v>39.01</v>
       </c>
       <c r="D21" t="n">
-        <v>47.42</v>
+        <v>47.62</v>
       </c>
       <c r="E21" t="n">
-        <v>-25.72</v>
+        <v>-26.59</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>SHREECEM</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>23855</v>
+      </c>
+      <c r="C22" t="n">
+        <v>39.06</v>
+      </c>
+      <c r="D22" t="n">
+        <v>42.43</v>
+      </c>
+      <c r="E22" t="n">
+        <v>-21.75</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ONGC</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>234.65</v>
+      </c>
+      <c r="C23" t="n">
+        <v>39.17</v>
+      </c>
+      <c r="D23" t="n">
+        <v>46.74</v>
+      </c>
+      <c r="E23" t="n">
+        <v>-22.15</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>DRREDDY</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1155</v>
+      </c>
+      <c r="C24" t="n">
+        <v>39.38</v>
+      </c>
+      <c r="D24" t="n">
+        <v>45.48</v>
+      </c>
+      <c r="E24" t="n">
+        <v>-16.04</v>
       </c>
     </row>
   </sheetData>

</xml_diff>